<commit_message>
[LZ004] tkinter GUI and frontend/backend integration finished.
</commit_message>
<xml_diff>
--- a/docx_xlsx_comparator/output/comparison_result.xlsx
+++ b/docx_xlsx_comparator/output/comparison_result.xlsx
@@ -432,10 +432,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.8" customWidth="1" min="1" max="1"/>
-    <col width="23.6" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="21.8" customWidth="1" min="3" max="3"/>
-    <col width="52.39999999999998" customWidth="1" min="4" max="4"/>
-    <col width="52.39999999999998" customWidth="1" min="5" max="5"/>
+    <col width="66.99999999999996" customWidth="1" min="4" max="4"/>
+    <col width="66.99999999999996" customWidth="1" min="5" max="5"/>
     <col width="12.8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
@@ -485,7 +485,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>建立帳號管理機制，包含帳號之申請、建立、修改、啟用、停用及刪除之程序。</t>
+          <t>應儲存與管理系統發展生命週期之相關文件。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -495,14 +495,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>帳號權限異動時填列申請表，並至後臺系統維護帳號資料。
-帳號申請、修改權限與停用均需經事先申請核可。</t>
+          <t>儲存及管理「程式規格書」、「系統管理手冊」、「使用者手冊」等文件，廠商於期末交付修訂版。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>帳號權限異動時填列申請表，並至後臺系統維護帳號資料。
-帳號申請、修改權限與停用均需經事先申請核可。</t>
+          <t>儲存及管理「程式規格書」、「系統管理手冊」、「使用者手冊」等文件，廠商於期末交付修訂版。</t>
         </is>
       </c>
       <c r="F2" t="b">
@@ -522,7 +520,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>資通系統閒置帳號應禁用。</t>
+          <t>使用密碼進行驗證時，應強制最低密碼複雜度；依機關密碼效期規定變更密碼。</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -532,12 +530,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>每半年之正式帳號清查，若超過半年未使用之帳號會將之停用。</t>
+          <t>使用者密碼長度須8碼，密碼內容須包含英文、數字及符號，每3個月須更新密碼。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>每半年之正式帳號清查，若超過半年未使用之帳號會將之停用。</t>
+          <t>使用者密碼長度須8碼，密碼內容須包含英文、數字及符號，每3個月須更新密碼。</t>
         </is>
       </c>
       <c r="F3" t="b">

</xml_diff>